<commit_message>
v9 patches: q20 broader detection (insults/rejections) + q21 reconciliation (agb_112, agb_081)
</commit_message>
<xml_diff>
--- a/Codebooks/LLM Codebook/LLM Coding - Audience Analysis.xlsx
+++ b/Codebooks/LLM Codebook/LLM Coding - Audience Analysis.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -483,7 +483,7 @@
       </c>
       <c r="B1" s="6" t="inlineStr">
         <is>
-          <t>v7 — final (post-recheck-audit patches applied)</t>
+          <t>v9 — final (post-recheck-audit-2 patches with broader q20 detection + q21 reconciliation)</t>
         </is>
       </c>
     </row>
@@ -519,7 +519,7 @@
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>b20e03f63866</t>
+          <t>54afeba8ae5f</t>
         </is>
       </c>
     </row>
@@ -611,7 +611,7 @@
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>Q4 keyword-level repair (gender words detected) • Q7-Other-Q7A gating • Q12→Q18 cross-check • Q20 correction-phrase regex • Q11 LLM repair for 4 stragglers • Methodology completed</t>
+          <t>v7 — Q4 keyword repair, Q7-Other-Q7A gating, Q12-&gt;Q18 cross-check, Q20 correction-phrase regex, Q11 LLM repair, Methodology completed</t>
         </is>
       </c>
     </row>
@@ -628,6 +628,18 @@
       <c r="B15" s="8" t="inlineStr">
         <is>
           <t>If reading via an external auditor, verify the SHA-256 above matches before commenting. ChatGPT/Claude responses cached on older versions of this file will report stale numbers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Audit fixes applied (v8)</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>v8 — Q20 broader pattern detection (insults + negations + explicit rejections); Q21=Yes but all sub-fields=No reconciled to Q21=No (AGB_112, AGB_081)</t>
         </is>
       </c>
     </row>
@@ -1436,7 +1448,7 @@
       </c>
       <c r="AP3" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="AQ3" s="2" t="inlineStr">
@@ -3798,10 +3810,14 @@
       <c r="AM15" s="2" t="n"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="AO15" s="2" t="n"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AO15" s="2" t="inlineStr">
+        <is>
+          <t>Disputes/rejects: "ith it,you too get sense walai"</t>
+        </is>
+      </c>
       <c r="AP15" s="2" t="inlineStr">
         <is>
           <t>No</t>
@@ -7364,7 +7380,7 @@
       <c r="AO33" s="2" t="n"/>
       <c r="AP33" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="AQ33" s="2" t="inlineStr">
@@ -8134,10 +8150,14 @@
       <c r="AM37" s="2" t="n"/>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="AO37" s="2" t="n"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AO37" s="2" t="inlineStr">
+        <is>
+          <t>Disputes/rejects: ", pretty posh. Nobody is glorifying cheating here. Have you ever asked yourself why m"</t>
+        </is>
+      </c>
       <c r="AP37" s="2" t="inlineStr">
         <is>
           <t>No</t>
@@ -42716,10 +42736,14 @@
       <c r="AM10" s="2" t="n"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="AO10" s="2" t="n"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AO10" s="2" t="inlineStr">
+        <is>
+          <t>Disputes/rejects: "Women are not cars you dumb toad!"</t>
+        </is>
+      </c>
       <c r="AP10" s="2" t="inlineStr">
         <is>
           <t>No</t>
@@ -46267,10 +46291,14 @@
       <c r="AM28" s="2" t="n"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="AO28" s="2" t="n"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AO28" s="2" t="inlineStr">
+        <is>
+          <t>Disputes/rejects: "Women are not cars so your line of reasoning is already questionable"</t>
+        </is>
+      </c>
       <c r="AP28" s="2" t="inlineStr">
         <is>
           <t>No</t>
@@ -47058,10 +47086,14 @@
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="AO32" s="2" t="n"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AO32" s="2" t="inlineStr">
+        <is>
+          <t>Disputes/rejects: "Men are not motorcycles with one headlamp.  Diversify, seduce fuck more w"</t>
+        </is>
+      </c>
       <c r="AP32" s="2" t="inlineStr">
         <is>
           <t>No</t>
@@ -47652,10 +47684,14 @@
       <c r="AM35" s="2" t="n"/>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="AO35" s="2" t="n"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AO35" s="2" t="inlineStr">
+        <is>
+          <t>Disputes/rejects: "Women are not cars"</t>
+        </is>
+      </c>
       <c r="AP35" s="2" t="inlineStr">
         <is>
           <t>No</t>
@@ -71394,10 +71430,14 @@
       </c>
       <c r="AN155" s="2" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="AO155" s="2" t="n"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AO155" s="2" t="inlineStr">
+        <is>
+          <t>Disputes/rejects: "ing black men, men are not machines they are human beings with emotions hence there s"</t>
+        </is>
+      </c>
       <c r="AP155" s="2" t="inlineStr">
         <is>
           <t>No</t>

</xml_diff>